<commit_message>
increased testing to allow agregated and granular comparisons
</commit_message>
<xml_diff>
--- a/tests/test_statistical_accuracy/data/demog_2023.xlsx
+++ b/tests/test_statistical_accuracy/data/demog_2023.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\philip.main\Source\dashboard-stats\tests\test_statistical_accuracy\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66D92885-46D4-4CDC-B60D-2CF59980FA0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{010754C1-F29E-4625-BE62-4AA71CFFE0F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="10240" xr2:uid="{988AF709-8AAF-41EE-8BA0-8AB60EF19A83}"/>
+    <workbookView xWindow="-28965" yWindow="-105" windowWidth="29130" windowHeight="15810" xr2:uid="{988AF709-8AAF-41EE-8BA0-8AB60EF19A83}"/>
   </bookViews>
   <sheets>
     <sheet name="CKD" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="71">
   <si>
     <t>Centre</t>
   </si>
@@ -76,9 +76,6 @@
     <t>% stage G5</t>
   </si>
   <si>
-    <t>Bangor</t>
-  </si>
-  <si>
     <t>Bham</t>
   </si>
   <si>
@@ -254,9 +251,6 @@
   </si>
   <si>
     <t>% with Tx</t>
-  </si>
-  <si>
-    <t>"</t>
   </si>
 </sst>
 </file>
@@ -628,7 +622,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84870F40-C8C8-4075-A648-2BFA53A7B634}">
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="10.08984375" bestFit="1" customWidth="1"/>
@@ -683,38 +677,38 @@
       <c r="A2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" t="s">
-        <v>72</v>
+      <c r="B2">
+        <v>1228</v>
       </c>
       <c r="C2">
-        <v>66.400000000000006</v>
+        <v>70.3</v>
       </c>
       <c r="D2">
-        <v>33.299999999999997</v>
+        <v>53.7</v>
       </c>
       <c r="E2">
-        <v>100</v>
+        <v>59.5</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>26.7</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>11.4</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="I2">
-        <v>66.7</v>
+        <v>11.1</v>
       </c>
       <c r="J2">
-        <v>25</v>
+        <v>13.9</v>
       </c>
       <c r="K2">
-        <v>14.3</v>
+        <v>6</v>
       </c>
       <c r="L2">
-        <v>40</v>
+        <v>33.6</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
@@ -722,37 +716,37 @@
         <v>13</v>
       </c>
       <c r="B3">
-        <v>1228</v>
+        <v>110</v>
       </c>
       <c r="C3">
-        <v>70.3</v>
+        <v>73.400000000000006</v>
       </c>
       <c r="D3">
-        <v>53.7</v>
+        <v>60.9</v>
       </c>
       <c r="E3">
-        <v>59.5</v>
+        <v>93.4</v>
       </c>
       <c r="F3">
-        <v>26.7</v>
+        <v>1.9</v>
       </c>
       <c r="G3">
-        <v>11.4</v>
+        <v>2.8</v>
       </c>
       <c r="H3">
-        <v>2.5</v>
+        <v>1.9</v>
       </c>
       <c r="I3">
-        <v>11.1</v>
+        <v>3.6</v>
       </c>
       <c r="J3">
-        <v>13.9</v>
+        <v>43.6</v>
       </c>
       <c r="K3">
-        <v>6</v>
+        <v>31.9</v>
       </c>
       <c r="L3">
-        <v>33.6</v>
+        <v>63.4</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
@@ -760,37 +754,37 @@
         <v>14</v>
       </c>
       <c r="B4">
-        <v>110</v>
+        <v>1024</v>
       </c>
       <c r="C4">
-        <v>73.400000000000006</v>
+        <v>74.599999999999994</v>
       </c>
       <c r="D4">
-        <v>60.9</v>
+        <v>58.8</v>
       </c>
       <c r="E4">
-        <v>93.4</v>
+        <v>93.2</v>
       </c>
       <c r="F4">
-        <v>1.9</v>
+        <v>4</v>
       </c>
       <c r="G4">
-        <v>2.8</v>
+        <v>1.7</v>
       </c>
       <c r="H4">
-        <v>1.9</v>
+        <v>1.2</v>
       </c>
       <c r="I4">
-        <v>3.6</v>
+        <v>35.799999999999997</v>
       </c>
       <c r="J4">
-        <v>43.6</v>
+        <v>71.5</v>
       </c>
       <c r="K4">
-        <v>31.9</v>
+        <v>66.900000000000006</v>
       </c>
       <c r="L4">
-        <v>63.4</v>
+        <v>86.9</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
@@ -798,37 +792,37 @@
         <v>15</v>
       </c>
       <c r="B5">
-        <v>1024</v>
+        <v>527</v>
       </c>
       <c r="C5">
-        <v>74.599999999999994</v>
+        <v>78.8</v>
       </c>
       <c r="D5">
-        <v>58.8</v>
+        <v>56.2</v>
       </c>
       <c r="E5">
-        <v>93.2</v>
+        <v>100</v>
       </c>
       <c r="F5">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>1.7</v>
+        <v>0</v>
       </c>
       <c r="H5">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="I5">
-        <v>35.799999999999997</v>
+        <v>39.299999999999997</v>
       </c>
       <c r="J5">
-        <v>71.5</v>
+        <v>15.9</v>
       </c>
       <c r="K5">
-        <v>66.900000000000006</v>
+        <v>11.9</v>
       </c>
       <c r="L5">
-        <v>86.9</v>
+        <v>32.1</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
@@ -836,13 +830,13 @@
         <v>16</v>
       </c>
       <c r="B6">
-        <v>527</v>
+        <v>19</v>
       </c>
       <c r="C6">
-        <v>78.8</v>
+        <v>79.400000000000006</v>
       </c>
       <c r="D6">
-        <v>56.2</v>
+        <v>68.400000000000006</v>
       </c>
       <c r="E6">
         <v>100</v>
@@ -857,16 +851,16 @@
         <v>0</v>
       </c>
       <c r="I6">
-        <v>39.299999999999997</v>
+        <v>47.4</v>
       </c>
       <c r="J6">
-        <v>15.9</v>
+        <v>42.1</v>
       </c>
       <c r="K6">
-        <v>11.9</v>
+        <v>33.299999999999997</v>
       </c>
       <c r="L6">
-        <v>32.1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
@@ -874,37 +868,37 @@
         <v>17</v>
       </c>
       <c r="B7">
-        <v>19</v>
+        <v>716</v>
       </c>
       <c r="C7">
-        <v>79.400000000000006</v>
+        <v>78.8</v>
       </c>
       <c r="D7">
-        <v>68.400000000000006</v>
+        <v>54.6</v>
       </c>
       <c r="E7">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>5.6</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>2.7</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="I7">
-        <v>47.4</v>
+        <v>13.3</v>
       </c>
       <c r="J7">
-        <v>42.1</v>
+        <v>96.8</v>
       </c>
       <c r="K7">
-        <v>33.299999999999997</v>
+        <v>96.5</v>
       </c>
       <c r="L7">
-        <v>50</v>
+        <v>97.9</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
@@ -912,37 +906,37 @@
         <v>18</v>
       </c>
       <c r="B8">
-        <v>716</v>
+        <v>1164</v>
       </c>
       <c r="C8">
-        <v>78.8</v>
+        <v>79.3</v>
       </c>
       <c r="D8">
-        <v>54.6</v>
+        <v>57.9</v>
       </c>
       <c r="E8">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="F8">
-        <v>5.6</v>
+        <v>2</v>
       </c>
       <c r="G8">
-        <v>2.7</v>
+        <v>1.7</v>
       </c>
       <c r="H8">
-        <v>0.6</v>
+        <v>1.3</v>
       </c>
       <c r="I8">
-        <v>13.3</v>
+        <v>7.2</v>
       </c>
       <c r="J8">
-        <v>96.8</v>
+        <v>48.5</v>
       </c>
       <c r="K8">
-        <v>96.5</v>
+        <v>46.8</v>
       </c>
       <c r="L8">
-        <v>97.9</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
@@ -950,37 +944,37 @@
         <v>19</v>
       </c>
       <c r="B9">
-        <v>1164</v>
+        <v>957</v>
       </c>
       <c r="C9">
-        <v>79.3</v>
+        <v>72.599999999999994</v>
       </c>
       <c r="D9">
-        <v>57.9</v>
+        <v>55.8</v>
       </c>
       <c r="E9">
-        <v>95</v>
+        <v>58</v>
       </c>
       <c r="F9">
-        <v>2</v>
+        <v>7.6</v>
       </c>
       <c r="G9">
-        <v>1.7</v>
+        <v>29.2</v>
       </c>
       <c r="H9">
-        <v>1.3</v>
+        <v>5.2</v>
       </c>
       <c r="I9">
-        <v>7.2</v>
+        <v>11.9</v>
       </c>
       <c r="J9">
-        <v>48.5</v>
+        <v>93.1</v>
       </c>
       <c r="K9">
-        <v>46.8</v>
+        <v>91.1</v>
       </c>
       <c r="L9">
-        <v>61</v>
+        <v>98.2</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
@@ -988,37 +982,37 @@
         <v>20</v>
       </c>
       <c r="B10">
-        <v>957</v>
+        <v>412</v>
       </c>
       <c r="C10">
-        <v>72.599999999999994</v>
+        <v>68.8</v>
       </c>
       <c r="D10">
-        <v>55.8</v>
+        <v>61.4</v>
       </c>
       <c r="E10">
-        <v>58</v>
+        <v>41.1</v>
       </c>
       <c r="F10">
-        <v>7.6</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="G10">
-        <v>29.2</v>
+        <v>47.2</v>
       </c>
       <c r="H10">
-        <v>5.2</v>
+        <v>3.6</v>
       </c>
       <c r="I10">
-        <v>11.9</v>
+        <v>31.6</v>
       </c>
       <c r="J10">
-        <v>93.1</v>
+        <v>5.6</v>
       </c>
       <c r="K10">
-        <v>91.1</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="L10">
-        <v>98.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
@@ -1026,37 +1020,37 @@
         <v>21</v>
       </c>
       <c r="B11">
-        <v>412</v>
+        <v>2693</v>
       </c>
       <c r="C11">
-        <v>68.8</v>
+        <v>76.7</v>
       </c>
       <c r="D11">
-        <v>61.4</v>
+        <v>56.8</v>
       </c>
       <c r="E11">
-        <v>41.1</v>
+        <v>55.5</v>
       </c>
       <c r="F11">
-        <v>8.1999999999999993</v>
+        <v>17.899999999999999</v>
       </c>
       <c r="G11">
-        <v>47.2</v>
+        <v>12.5</v>
       </c>
       <c r="H11">
-        <v>3.6</v>
+        <v>14.2</v>
       </c>
       <c r="I11">
-        <v>31.6</v>
+        <v>11.4</v>
       </c>
       <c r="J11">
-        <v>5.6</v>
+        <v>41.3</v>
       </c>
       <c r="K11">
-        <v>5.0999999999999996</v>
+        <v>37.4</v>
       </c>
       <c r="L11">
-        <v>6</v>
+        <v>52.7</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
@@ -1064,37 +1058,37 @@
         <v>22</v>
       </c>
       <c r="B12">
-        <v>2693</v>
+        <v>4146</v>
       </c>
       <c r="C12">
-        <v>76.7</v>
+        <v>78.099999999999994</v>
       </c>
       <c r="D12">
-        <v>56.8</v>
+        <v>54.4</v>
       </c>
       <c r="E12">
-        <v>55.5</v>
+        <v>77.599999999999994</v>
       </c>
       <c r="F12">
-        <v>17.899999999999999</v>
+        <v>17.5</v>
       </c>
       <c r="G12">
-        <v>12.5</v>
+        <v>3.4</v>
       </c>
       <c r="H12">
-        <v>14.2</v>
+        <v>1.6</v>
       </c>
       <c r="I12">
-        <v>11.4</v>
+        <v>27.3</v>
       </c>
       <c r="J12">
-        <v>41.3</v>
+        <v>55.6</v>
       </c>
       <c r="K12">
-        <v>37.4</v>
+        <v>53.8</v>
       </c>
       <c r="L12">
-        <v>52.7</v>
+        <v>64.400000000000006</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
@@ -1102,37 +1096,37 @@
         <v>23</v>
       </c>
       <c r="B13">
-        <v>4146</v>
+        <v>594</v>
       </c>
       <c r="C13">
-        <v>78.099999999999994</v>
+        <v>73</v>
       </c>
       <c r="D13">
-        <v>54.4</v>
+        <v>57.6</v>
       </c>
       <c r="E13">
-        <v>77.599999999999994</v>
+        <v>94.5</v>
       </c>
       <c r="F13">
-        <v>17.5</v>
+        <v>3</v>
       </c>
       <c r="G13">
-        <v>3.4</v>
+        <v>0.9</v>
       </c>
       <c r="H13">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="I13">
-        <v>27.3</v>
+        <v>20.9</v>
       </c>
       <c r="J13">
-        <v>55.6</v>
+        <v>25.3</v>
       </c>
       <c r="K13">
-        <v>53.8</v>
+        <v>19</v>
       </c>
       <c r="L13">
-        <v>64.400000000000006</v>
+        <v>39.299999999999997</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
@@ -1140,37 +1134,37 @@
         <v>24</v>
       </c>
       <c r="B14">
-        <v>594</v>
+        <v>529</v>
       </c>
       <c r="C14">
-        <v>73</v>
+        <v>72.7</v>
       </c>
       <c r="D14">
-        <v>57.6</v>
+        <v>58.2</v>
       </c>
       <c r="E14">
-        <v>94.5</v>
+        <v>84.8</v>
       </c>
       <c r="F14">
-        <v>3</v>
+        <v>5.9</v>
       </c>
       <c r="G14">
-        <v>0.9</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="H14">
-        <v>1.7</v>
+        <v>4.7</v>
       </c>
       <c r="I14">
-        <v>20.9</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="J14">
-        <v>25.3</v>
+        <v>83.9</v>
       </c>
       <c r="K14">
-        <v>19</v>
+        <v>83.2</v>
       </c>
       <c r="L14">
-        <v>39.299999999999997</v>
+        <v>84.5</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
@@ -1178,37 +1172,37 @@
         <v>25</v>
       </c>
       <c r="B15">
-        <v>529</v>
+        <v>1523</v>
       </c>
       <c r="C15">
-        <v>72.7</v>
+        <v>75.099999999999994</v>
       </c>
       <c r="D15">
-        <v>58.2</v>
+        <v>60.7</v>
       </c>
       <c r="E15">
-        <v>84.8</v>
+        <v>85.6</v>
       </c>
       <c r="F15">
-        <v>5.9</v>
+        <v>7.8</v>
       </c>
       <c r="G15">
-        <v>4.5999999999999996</v>
+        <v>3.4</v>
       </c>
       <c r="H15">
-        <v>4.7</v>
+        <v>3.2</v>
       </c>
       <c r="I15">
-        <v>4.4000000000000004</v>
+        <v>19.600000000000001</v>
       </c>
       <c r="J15">
-        <v>83.9</v>
+        <v>20.7</v>
       </c>
       <c r="K15">
-        <v>83.2</v>
+        <v>16.5</v>
       </c>
       <c r="L15">
-        <v>84.5</v>
+        <v>33.4</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
@@ -1216,37 +1210,37 @@
         <v>26</v>
       </c>
       <c r="B16">
-        <v>1523</v>
+        <v>949</v>
       </c>
       <c r="C16">
-        <v>75.099999999999994</v>
+        <v>79.099999999999994</v>
       </c>
       <c r="D16">
-        <v>60.7</v>
+        <v>54.5</v>
       </c>
       <c r="E16">
-        <v>85.6</v>
+        <v>98.7</v>
       </c>
       <c r="F16">
-        <v>7.8</v>
+        <v>0.1</v>
       </c>
       <c r="G16">
-        <v>3.4</v>
+        <v>0.2</v>
       </c>
       <c r="H16">
-        <v>3.2</v>
+        <v>1</v>
       </c>
       <c r="I16">
-        <v>19.600000000000001</v>
+        <v>6.4</v>
       </c>
       <c r="J16">
-        <v>20.7</v>
+        <v>13.7</v>
       </c>
       <c r="K16">
-        <v>16.5</v>
+        <v>13.5</v>
       </c>
       <c r="L16">
-        <v>33.4</v>
+        <v>14.6</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.35">
@@ -1254,37 +1248,37 @@
         <v>27</v>
       </c>
       <c r="B17">
-        <v>949</v>
+        <v>2127</v>
       </c>
       <c r="C17">
-        <v>79.099999999999994</v>
+        <v>76.3</v>
       </c>
       <c r="D17">
-        <v>54.5</v>
+        <v>59.3</v>
       </c>
       <c r="E17">
-        <v>98.7</v>
+        <v>97.7</v>
       </c>
       <c r="F17">
-        <v>0.1</v>
+        <v>1.3</v>
       </c>
       <c r="G17">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="H17">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I17">
-        <v>6.4</v>
+        <v>43.9</v>
       </c>
       <c r="J17">
-        <v>13.7</v>
+        <v>8.4</v>
       </c>
       <c r="K17">
-        <v>13.5</v>
+        <v>6.5</v>
       </c>
       <c r="L17">
-        <v>14.6</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.35">
@@ -1292,37 +1286,37 @@
         <v>28</v>
       </c>
       <c r="B18">
-        <v>2127</v>
+        <v>2824</v>
       </c>
       <c r="C18">
-        <v>76.3</v>
+        <v>78.400000000000006</v>
       </c>
       <c r="D18">
-        <v>59.3</v>
+        <v>54.6</v>
       </c>
       <c r="E18">
-        <v>97.7</v>
+        <v>89.6</v>
       </c>
       <c r="F18">
-        <v>1.3</v>
+        <v>7.4</v>
       </c>
       <c r="G18">
-        <v>0.4</v>
+        <v>2</v>
       </c>
       <c r="H18">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="I18">
-        <v>43.9</v>
+        <v>51.8</v>
       </c>
       <c r="J18">
-        <v>8.4</v>
+        <v>3.4</v>
       </c>
       <c r="K18">
-        <v>6.5</v>
+        <v>2.8</v>
       </c>
       <c r="L18">
-        <v>13.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.35">
@@ -1330,37 +1324,37 @@
         <v>29</v>
       </c>
       <c r="B19">
-        <v>2824</v>
+        <v>443</v>
       </c>
       <c r="C19">
-        <v>78.400000000000006</v>
+        <v>75.5</v>
       </c>
       <c r="D19">
-        <v>54.6</v>
+        <v>64.599999999999994</v>
       </c>
       <c r="E19">
-        <v>89.6</v>
+        <v>67.400000000000006</v>
       </c>
       <c r="F19">
-        <v>7.4</v>
+        <v>13.5</v>
       </c>
       <c r="G19">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="H19">
-        <v>1</v>
+        <v>16.7</v>
       </c>
       <c r="I19">
-        <v>51.8</v>
+        <v>44.7</v>
       </c>
       <c r="J19">
-        <v>3.4</v>
+        <v>73.099999999999994</v>
       </c>
       <c r="K19">
-        <v>2.8</v>
+        <v>55.7</v>
       </c>
       <c r="L19">
-        <v>6</v>
+        <v>96.3</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.35">
@@ -1368,37 +1362,37 @@
         <v>30</v>
       </c>
       <c r="B20">
-        <v>443</v>
+        <v>774</v>
       </c>
       <c r="C20">
-        <v>75.5</v>
+        <v>75.099999999999994</v>
       </c>
       <c r="D20">
-        <v>64.599999999999994</v>
+        <v>56.7</v>
       </c>
       <c r="E20">
-        <v>67.400000000000006</v>
+        <v>83.7</v>
       </c>
       <c r="F20">
-        <v>13.5</v>
+        <v>10.5</v>
       </c>
       <c r="G20">
-        <v>2.5</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="H20">
-        <v>16.7</v>
+        <v>1.4</v>
       </c>
       <c r="I20">
-        <v>44.7</v>
+        <v>35.799999999999997</v>
       </c>
       <c r="J20">
-        <v>73.099999999999994</v>
+        <v>8.1</v>
       </c>
       <c r="K20">
-        <v>55.7</v>
+        <v>7.7</v>
       </c>
       <c r="L20">
-        <v>96.3</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.35">
@@ -1406,37 +1400,37 @@
         <v>31</v>
       </c>
       <c r="B21">
-        <v>774</v>
+        <v>396</v>
       </c>
       <c r="C21">
-        <v>75.099999999999994</v>
+        <v>67.5</v>
       </c>
       <c r="D21">
-        <v>56.7</v>
+        <v>57.1</v>
       </c>
       <c r="E21">
-        <v>83.7</v>
+        <v>84.6</v>
       </c>
       <c r="F21">
-        <v>10.5</v>
+        <v>8.1</v>
       </c>
       <c r="G21">
-        <v>4.4000000000000004</v>
+        <v>3.9</v>
       </c>
       <c r="H21">
-        <v>1.4</v>
+        <v>3.4</v>
       </c>
       <c r="I21">
-        <v>35.799999999999997</v>
+        <v>3.3</v>
       </c>
       <c r="J21">
-        <v>8.1</v>
+        <v>99.2</v>
       </c>
       <c r="K21">
-        <v>7.7</v>
+        <v>99.1</v>
       </c>
       <c r="L21">
-        <v>11.1</v>
+        <v>99.4</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.35">
@@ -1444,37 +1438,37 @@
         <v>32</v>
       </c>
       <c r="B22">
-        <v>396</v>
+        <v>2102</v>
       </c>
       <c r="C22">
-        <v>67.5</v>
+        <v>79.3</v>
       </c>
       <c r="D22">
-        <v>57.1</v>
+        <v>54.3</v>
       </c>
       <c r="E22">
-        <v>84.6</v>
+        <v>98.3</v>
       </c>
       <c r="F22">
-        <v>8.1</v>
+        <v>0.7</v>
       </c>
       <c r="G22">
-        <v>3.9</v>
+        <v>0.6</v>
       </c>
       <c r="H22">
-        <v>3.4</v>
+        <v>0.4</v>
       </c>
       <c r="I22">
-        <v>3.3</v>
+        <v>42.9</v>
       </c>
       <c r="J22">
-        <v>99.2</v>
+        <v>34.6</v>
       </c>
       <c r="K22">
-        <v>99.1</v>
+        <v>31.9</v>
       </c>
       <c r="L22">
-        <v>99.4</v>
+        <v>49.3</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.35">
@@ -1482,37 +1476,37 @@
         <v>33</v>
       </c>
       <c r="B23">
-        <v>2102</v>
+        <v>869</v>
       </c>
       <c r="C23">
-        <v>79.3</v>
+        <v>79.599999999999994</v>
       </c>
       <c r="D23">
-        <v>54.3</v>
+        <v>57.3</v>
       </c>
       <c r="E23">
-        <v>98.3</v>
+        <v>99.3</v>
       </c>
       <c r="F23">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="G23">
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
       <c r="H23">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="I23">
-        <v>42.9</v>
+        <v>0.5</v>
       </c>
       <c r="J23">
-        <v>34.6</v>
+        <v>22.7</v>
       </c>
       <c r="K23">
-        <v>31.9</v>
+        <v>18.3</v>
       </c>
       <c r="L23">
-        <v>49.3</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.35">
@@ -1520,74 +1514,36 @@
         <v>34</v>
       </c>
       <c r="B24">
-        <v>869</v>
+        <v>135</v>
       </c>
       <c r="C24">
-        <v>79.599999999999994</v>
+        <v>78.2</v>
       </c>
       <c r="D24">
-        <v>57.3</v>
+        <v>60</v>
       </c>
       <c r="E24">
-        <v>99.3</v>
+        <v>100</v>
       </c>
       <c r="F24">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="G24">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="H24">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="I24">
-        <v>0.5</v>
+        <v>63</v>
       </c>
       <c r="J24">
-        <v>22.7</v>
+        <v>21.5</v>
       </c>
       <c r="K24">
-        <v>18.3</v>
+        <v>14.3</v>
       </c>
       <c r="L24">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>35</v>
-      </c>
-      <c r="B25">
-        <v>135</v>
-      </c>
-      <c r="C25">
-        <v>78.2</v>
-      </c>
-      <c r="D25">
-        <v>60</v>
-      </c>
-      <c r="E25">
-        <v>100</v>
-      </c>
-      <c r="F25">
-        <v>0</v>
-      </c>
-      <c r="G25">
-        <v>0</v>
-      </c>
-      <c r="H25">
-        <v>0</v>
-      </c>
-      <c r="I25">
-        <v>63</v>
-      </c>
-      <c r="J25">
-        <v>21.5</v>
-      </c>
-      <c r="K25">
-        <v>14.3</v>
-      </c>
-      <c r="L25">
         <v>40.5</v>
       </c>
     </row>
@@ -1616,22 +1572,22 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" t="s">
         <v>36</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>37</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>38</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>39</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>40</v>
-      </c>
-      <c r="G1" t="s">
-        <v>41</v>
       </c>
       <c r="H1" t="s">
         <v>2</v>
@@ -1657,7 +1613,7 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B2">
         <v>367</v>
@@ -1701,7 +1657,7 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3">
         <v>101</v>
@@ -1745,7 +1701,7 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4">
         <v>157</v>
@@ -1789,7 +1745,7 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5">
         <v>172</v>
@@ -1833,7 +1789,7 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6">
         <v>87</v>
@@ -1877,7 +1833,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7">
         <v>45</v>
@@ -1921,7 +1877,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B8">
         <v>320</v>
@@ -1965,7 +1921,7 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B9">
         <v>47</v>
@@ -2009,7 +1965,7 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B10">
         <v>131</v>
@@ -2053,7 +2009,7 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B11">
         <v>109</v>
@@ -2097,7 +2053,7 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B12">
         <v>71</v>
@@ -2141,7 +2097,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B13">
         <v>98</v>
@@ -2185,7 +2141,7 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B14">
         <v>49</v>
@@ -2229,7 +2185,7 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B15">
         <v>210</v>
@@ -2273,7 +2229,7 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B16">
         <v>150</v>
@@ -2293,7 +2249,7 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B17">
         <v>84</v>
@@ -2337,7 +2293,7 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B18">
         <v>119</v>
@@ -2381,7 +2337,7 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B19">
         <v>42</v>
@@ -2425,7 +2381,7 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B20">
         <v>163</v>
@@ -2469,7 +2425,7 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B21">
         <v>348</v>
@@ -2513,7 +2469,7 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B22">
         <v>164</v>
@@ -2557,7 +2513,7 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B23">
         <v>157</v>
@@ -2601,7 +2557,7 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B24">
         <v>265</v>
@@ -2645,7 +2601,7 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B25">
         <v>88</v>
@@ -2689,7 +2645,7 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B26">
         <v>390</v>
@@ -2733,7 +2689,7 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B27">
         <v>179</v>
@@ -2777,7 +2733,7 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B28">
         <v>357</v>
@@ -2821,7 +2777,7 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B29">
         <v>160</v>
@@ -2865,7 +2821,7 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B30">
         <v>205</v>
@@ -2885,7 +2841,7 @@
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B31">
         <v>111</v>
@@ -2929,7 +2885,7 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B32">
         <v>155</v>
@@ -2973,7 +2929,7 @@
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B33">
         <v>75</v>
@@ -3017,7 +2973,7 @@
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B34">
         <v>109</v>
@@ -3061,7 +3017,7 @@
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B35">
         <v>221</v>
@@ -3105,7 +3061,7 @@
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B36">
         <v>61</v>
@@ -3149,7 +3105,7 @@
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B37">
         <v>241</v>
@@ -3181,7 +3137,7 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B38">
         <v>198</v>
@@ -3225,7 +3181,7 @@
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B39">
         <v>132</v>
@@ -3269,7 +3225,7 @@
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B40">
         <v>198</v>
@@ -3313,7 +3269,7 @@
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B41">
         <v>164</v>
@@ -3357,7 +3313,7 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B42">
         <v>63</v>
@@ -3401,7 +3357,7 @@
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B43">
         <v>173</v>
@@ -3445,7 +3401,7 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B44">
         <v>121</v>
@@ -3489,7 +3445,7 @@
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B45">
         <v>76</v>
@@ -3533,7 +3489,7 @@
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B46">
         <v>58</v>
@@ -3577,7 +3533,7 @@
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B47">
         <v>40</v>
@@ -3621,7 +3577,7 @@
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B48">
         <v>139</v>
@@ -3665,7 +3621,7 @@
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B49">
         <v>46</v>
@@ -3730,19 +3686,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" t="s">
         <v>36</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>37</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>38</v>
       </c>
-      <c r="E1" t="s">
-        <v>39</v>
-      </c>
       <c r="F1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G1" t="s">
         <v>2</v>
@@ -3768,7 +3724,7 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B2">
         <v>3417</v>
@@ -3809,7 +3765,7 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3">
         <v>824</v>
@@ -3850,7 +3806,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4">
         <v>1145</v>
@@ -3891,7 +3847,7 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5">
         <v>1522</v>
@@ -3932,7 +3888,7 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6">
         <v>1629</v>
@@ -3973,7 +3929,7 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7">
         <v>305</v>
@@ -4014,7 +3970,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B8">
         <v>2001</v>
@@ -4055,7 +4011,7 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B9">
         <v>164</v>
@@ -4096,7 +4052,7 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B10">
         <v>1158</v>
@@ -4137,7 +4093,7 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B11">
         <v>735</v>
@@ -4178,7 +4134,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B12">
         <v>387</v>
@@ -4219,7 +4175,7 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B13">
         <v>816</v>
@@ -4260,7 +4216,7 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B14">
         <v>368</v>
@@ -4301,7 +4257,7 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B15">
         <v>974</v>
@@ -4342,7 +4298,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B16">
         <v>1127</v>
@@ -4362,7 +4318,7 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B17">
         <v>560</v>
@@ -4403,7 +4359,7 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B18">
         <v>959</v>
@@ -4444,7 +4400,7 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B19">
         <v>397</v>
@@ -4485,7 +4441,7 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B20">
         <v>1240</v>
@@ -4526,7 +4482,7 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B21">
         <v>2959</v>
@@ -4567,7 +4523,7 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B22">
         <v>2318</v>
@@ -4608,7 +4564,7 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B23">
         <v>1389</v>
@@ -4649,7 +4605,7 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B24">
         <v>2475</v>
@@ -4690,7 +4646,7 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B25">
         <v>878</v>
@@ -4731,7 +4687,7 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B26">
         <v>3681</v>
@@ -4772,7 +4728,7 @@
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B27">
         <v>1906</v>
@@ -4813,7 +4769,7 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B28">
         <v>2820</v>
@@ -4854,7 +4810,7 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B29">
         <v>1503</v>
@@ -4895,7 +4851,7 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B30">
         <v>2258</v>
@@ -4915,7 +4871,7 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B31">
         <v>971</v>
@@ -4956,7 +4912,7 @@
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B32">
         <v>1287</v>
@@ -4997,7 +4953,7 @@
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B33">
         <v>808</v>
@@ -5038,7 +4994,7 @@
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B34">
         <v>1195</v>
@@ -5079,7 +5035,7 @@
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B35">
         <v>2132</v>
@@ -5120,7 +5076,7 @@
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B36">
         <v>549</v>
@@ -5161,7 +5117,7 @@
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B37">
         <v>2030</v>
@@ -5202,7 +5158,7 @@
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B38">
         <v>1436</v>
@@ -5243,7 +5199,7 @@
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B39">
         <v>994</v>
@@ -5284,7 +5240,7 @@
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B40">
         <v>1371</v>
@@ -5325,7 +5281,7 @@
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B41">
         <v>1478</v>
@@ -5366,7 +5322,7 @@
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B42">
         <v>461</v>
@@ -5407,7 +5363,7 @@
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B43">
         <v>1117</v>
@@ -5448,7 +5404,7 @@
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B44">
         <v>921</v>
@@ -5489,7 +5445,7 @@
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B45">
         <v>590</v>
@@ -5530,7 +5486,7 @@
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B46">
         <v>468</v>
@@ -5571,7 +5527,7 @@
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B47">
         <v>387</v>
@@ -5612,7 +5568,7 @@
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B48">
         <v>780</v>
@@ -5653,7 +5609,7 @@
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B49">
         <v>610</v>

</xml_diff>